<commit_message>
feat: implement Leg1 optimization modules, APIs, and rollout planning interfaces for admin, district, and DFPD roles
</commit_message>
<xml_diff>
--- a/pds_admin_Punjab_R/Backend/Backend/Data_1.xlsx
+++ b/pds_admin_Punjab_R/Backend/Backend/Data_1.xlsx
@@ -23000,7 +23000,7 @@
     <t>SHRI SHIV KIRPA RICE MILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">SHRI BALAJI RICE INDUSTRIES  103404 </t>
+    <t>SHRI BALAJI RICE INDUSTRIES( 103404)</t>
   </si>
   <si>
     <t>Sudama Rice mill</t>
@@ -23171,7 +23171,7 @@
     <t>R K AGRO FOODS</t>
   </si>
   <si>
-    <t xml:space="preserve">SHRI GANESH RICE MILLS  102590 </t>
+    <t>SHRI GANESH RICE MILLS (102590)</t>
   </si>
   <si>
     <t>AGGARWAL RICE AND GEN MILLSBHAGTA BHAIKA</t>
@@ -23201,7 +23201,7 @@
     <t>SHREE BHAGAT JI RICE MILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">LAKSHAY RICE MILLS  105163 </t>
+    <t>LAKSHAY RICE MILLS (105163)</t>
   </si>
   <si>
     <t>GRAND RICE MILL</t>
@@ -23252,13 +23252,13 @@
     <t>DASHMESH RICE MILL</t>
   </si>
   <si>
-    <t xml:space="preserve">SHREE GANESHA RICE MILLS  101869 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SHREE KRIPALU RICE MILLS  101874 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SHREE MANGALMURTI RICE MILLS  101875 </t>
+    <t>SHREE GANESHA RICE MILLS (101869)</t>
+  </si>
+  <si>
+    <t>SHREE KRIPALU RICE MILLS (101874)</t>
+  </si>
+  <si>
+    <t>SHREE MANGALMURTI RICE MILLS (101875)</t>
   </si>
   <si>
     <t>SHREE GANPATI RICE MILLS</t>
@@ -23315,7 +23315,7 @@
     <t>BAHIARICEMILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">GOBIND RICE AND GENERAL MILLS  102501 </t>
+    <t>GOBIND RICE AND GENERAL MILLS (102501)</t>
   </si>
   <si>
     <t>HARIOM RICE MILLS</t>
@@ -23348,7 +23348,7 @@
     <t>SHYAM RICE MILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">AGGARWAL RICE MILLS  102829 </t>
+    <t>AGGARWAL RICE MILLS (102829)</t>
   </si>
   <si>
     <t>BEST RICE MILLS</t>
@@ -23357,7 +23357,7 @@
     <t>RP RICE MILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">SINGLA RICE MILLS  102915 </t>
+    <t>SINGLA RICE MILLS (102915)</t>
   </si>
   <si>
     <t>A.G RICE MILL</t>
@@ -23381,7 +23381,7 @@
     <t>SIDHI VINAYAK RICE AND GENERAL MILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">BHAGWATI COTSPIN  103613 </t>
+    <t>BHAGWATI COTSPIN (103613)</t>
   </si>
   <si>
     <t>SHREE BALAJI COTTON AND RICE MILLS</t>
@@ -23393,7 +23393,7 @@
     <t>PARDEEP RICE MILLS UNIT II</t>
   </si>
   <si>
-    <t xml:space="preserve">A.S.RICE MILLS  104276 </t>
+    <t>A.S.RICE MILLS (104276)</t>
   </si>
   <si>
     <t>PUNJABI AGRO RICE MILLS</t>
@@ -23432,10 +23432,10 @@
     <t>ADC HEALTH FOOD</t>
   </si>
   <si>
-    <t xml:space="preserve">WAHEGURU RICE MILLS  100670 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">DHILLON AGRO FOODS  100679 </t>
+    <t>WAHEGURU RICE MILLS (100670)</t>
+  </si>
+  <si>
+    <t>DHILLON AGRO FOODS (100679)</t>
   </si>
   <si>
     <t>RAM RICE MILL</t>
@@ -23534,7 +23534,7 @@
     <t>Shri Mahadev Rice Mills</t>
   </si>
   <si>
-    <t xml:space="preserve">Nirwair Rice &amp; General Mills  106420 </t>
+    <t>Nirwair Rice &amp; General Mills (106420)</t>
   </si>
   <si>
     <t>Goniana Rice Mills</t>
@@ -23561,7 +23561,7 @@
     <t>SHRI LUXMI RICE MILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">SHAM SUNDER RICE MILL  101547 </t>
+    <t>SHAM SUNDER RICE MILL (101547)</t>
   </si>
   <si>
     <t>RAMA KRISHNA RICE MILL</t>
@@ -23714,7 +23714,7 @@
     <t>SHRI KRISHNA RICE AND GENERAL MILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">SARASWATI RICE MILLS  101895 </t>
+    <t>SARASWATI RICE MILLS (101895)</t>
   </si>
   <si>
     <t>VARDHMAN RICE MILLS</t>
@@ -23777,7 +23777,7 @@
     <t>VARDHMAN JAIN RICE MILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">SHYAM AGRO FOODS  104572 </t>
+    <t>SHYAM AGRO FOODS (104572)</t>
   </si>
   <si>
     <t>SHREE RATTAN INDUSTRIES</t>
@@ -23846,7 +23846,7 @@
     <t>D.P.AGRO</t>
   </si>
   <si>
-    <t xml:space="preserve">SHRI GURDEV RICE MILL, RAMAN  107202 </t>
+    <t>SHRI GURDEV RICE MILL, RAMAN (107202)</t>
   </si>
   <si>
     <t>SATYAM RICE AND GENERAL MILL</t>
@@ -23990,7 +23990,7 @@
     <t>SATLUJ RICE MILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">SUGHRU MAL DHRAM RAJ RICE MILLS  102466 </t>
+    <t>SUGHRU MAL DHRAM RAJ RICE MILLS (102466)</t>
   </si>
   <si>
     <t>PUNJAB RICE MILL</t>
@@ -24077,7 +24077,7 @@
     <t>G.B RICE MILLS BHAIRUPA</t>
   </si>
   <si>
-    <t xml:space="preserve">MAHAVIR RICE MILLS, MEHRAJ  103029 </t>
+    <t>MAHAVIR RICE MILLS, MEHRAJ (103029)</t>
   </si>
   <si>
     <t>DHILLON OILS AND FATS PVT. LTD</t>
@@ -24089,7 +24089,7 @@
     <t>KULDEEP RICE  GENERAL MILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">SHRI GANESH RICE MILL  103086 </t>
+    <t>SHRI GANESH RICE MILL (103086)</t>
   </si>
   <si>
     <t>MAA DURGA RICE MILLS UNIT II</t>
@@ -24107,10 +24107,10 @@
     <t>BANSAL RICE MILL UNITII</t>
   </si>
   <si>
-    <t xml:space="preserve">RADHE KRISHNA RICE &amp; GINNING MILLS  103133 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">PARSHOTAM LAL RICE MILLS  103164 </t>
+    <t>RADHE KRISHNA RICE &amp; GINNING MILLS (103133)</t>
+  </si>
+  <si>
+    <t>PARSHOTAM LAL RICE MILLS (103164)</t>
   </si>
   <si>
     <t>SAHARA RICE GRAM UDYOG SAMITI</t>
@@ -24248,7 +24248,7 @@
     <t>SHRI HARI ANAND RICE MILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">Chiranji Lal Bhim Sain Rice Mills  108846 </t>
+    <t>Chiranji Lal Bhim Sain Rice Mills (108846)</t>
   </si>
   <si>
     <t>NAND RICE MILLS</t>
@@ -24290,10 +24290,10 @@
     <t>BANKEY BIHARI AGRO INDUSTRIES, MEHTA</t>
   </si>
   <si>
-    <t xml:space="preserve">Shree Ganesh Rice Mills  105813 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shree Gobind Rice Mills  105823 </t>
+    <t>Shree Ganesh Rice Mills (105813)</t>
+  </si>
+  <si>
+    <t>Shree Gobind Rice Mills (105823)</t>
   </si>
   <si>
     <t>JAI BHIKSHU RICE MILLS</t>
@@ -24320,7 +24320,7 @@
     <t>BJB RICE MILLS</t>
   </si>
   <si>
-    <t xml:space="preserve">Saraswati Agro Foods  106842 </t>
+    <t>Saraswati Agro Foods (106842)</t>
   </si>
   <si>
     <t>KARNI KIRPA RICE MILLS</t>

</xml_diff>